<commit_message>
added flowmeter sizing and fixed some bugs
</commit_message>
<xml_diff>
--- a/templates/IL.xlsx
+++ b/templates/IL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CIS_Automation\Program_v0.2\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20950280-BA05-4B42-9CB9-A8798FDC4FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C6E049-2173-4E6A-811E-C010ABA56998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="7" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
   <si>
     <t>CLIENT :</t>
   </si>
@@ -295,6 +295,9 @@
   <si>
     <t>Location:</t>
   </si>
+  <si>
+    <t>✓</t>
+  </si>
 </sst>
 </file>
 
@@ -303,7 +306,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14009]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -390,6 +393,12 @@
       <sz val="11"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Amasis MT Pro Black"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="16">
@@ -768,7 +777,7 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -909,15 +918,6 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -967,6 +967,14 @@
     </xf>
     <xf numFmtId="14" fontId="9" fillId="13" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1159,8 +1167,8 @@
       <xdr:rowOff>92165</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>571499</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>114299</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>534984</xdr:rowOff>
     </xdr:to>
@@ -1212,23 +1220,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1570,23 +1561,27 @@
     <col min="4" max="4" width="4.77734375" style="14" customWidth="1"/>
     <col min="5" max="5" width="7.21875" style="14" customWidth="1"/>
     <col min="6" max="6" width="5.77734375" style="14" customWidth="1"/>
-    <col min="7" max="7" width="4.5546875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="2.77734375" style="14" customWidth="1"/>
     <col min="8" max="8" width="5.44140625" style="14" customWidth="1"/>
     <col min="9" max="9" width="5.21875" style="14" customWidth="1"/>
     <col min="10" max="10" width="2.77734375" style="14" customWidth="1"/>
     <col min="11" max="11" width="5.77734375" style="14" customWidth="1"/>
     <col min="12" max="12" width="3.77734375" style="14" customWidth="1"/>
     <col min="13" max="13" width="4.21875" style="14" customWidth="1"/>
-    <col min="14" max="15" width="3.77734375" style="14" customWidth="1"/>
+    <col min="14" max="14" width="2.77734375" style="14" customWidth="1"/>
+    <col min="15" max="15" width="3.77734375" style="14" customWidth="1"/>
     <col min="16" max="16" width="6.21875" style="14" customWidth="1"/>
     <col min="17" max="17" width="4.77734375" style="14" customWidth="1"/>
-    <col min="18" max="20" width="3.77734375" style="14" customWidth="1"/>
+    <col min="18" max="18" width="2.77734375" style="14" customWidth="1"/>
+    <col min="19" max="20" width="3.77734375" style="14" customWidth="1"/>
     <col min="21" max="21" width="8.5546875" style="14" customWidth="1"/>
-    <col min="22" max="24" width="3.77734375" style="14" customWidth="1"/>
+    <col min="22" max="22" width="3.77734375" style="14" customWidth="1"/>
+    <col min="23" max="23" width="2.77734375" style="14" customWidth="1"/>
+    <col min="24" max="24" width="3.77734375" style="14" customWidth="1"/>
     <col min="25" max="25" width="5.21875" style="14" customWidth="1"/>
     <col min="26" max="26" width="6.21875" style="14" customWidth="1"/>
     <col min="27" max="27" width="5.77734375" style="14" customWidth="1"/>
-    <col min="28" max="28" width="3.77734375" style="14" customWidth="1"/>
+    <col min="28" max="28" width="2.77734375" style="14" customWidth="1"/>
     <col min="29" max="29" width="7" style="14" customWidth="1"/>
     <col min="30" max="30" width="3.77734375" style="14" customWidth="1"/>
     <col min="31" max="31" width="7.77734375" style="14" customWidth="1"/>
@@ -1600,7 +1595,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="55" t="s">
         <v>54</v>
       </c>
       <c r="B1" s="12"/>
@@ -1636,7 +1631,7 @@
       <c r="AF1" s="13"/>
     </row>
     <row r="2" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="55"/>
+      <c r="A2" s="56"/>
       <c r="B2" s="15"/>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -1670,35 +1665,35 @@
       <c r="AF2" s="16"/>
     </row>
     <row r="3" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="55"/>
+      <c r="A3" s="56"/>
       <c r="B3" s="17"/>
       <c r="AE3" s="16"/>
       <c r="AF3" s="16"/>
     </row>
     <row r="4" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="55"/>
+      <c r="A4" s="56"/>
       <c r="B4" s="17"/>
       <c r="AE4" s="16"/>
       <c r="AF4" s="16"/>
     </row>
     <row r="5" spans="1:35" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="55"/>
+      <c r="A5" s="56"/>
       <c r="B5" s="17"/>
       <c r="AE5" s="16"/>
       <c r="AF5" s="16"/>
     </row>
     <row r="6" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="55"/>
+      <c r="A6" s="56"/>
       <c r="B6" s="17"/>
       <c r="AE6" s="16"/>
       <c r="AF6" s="16"/>
       <c r="AH6" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="52"/>
     </row>
     <row r="7" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="55"/>
+      <c r="A7" s="56"/>
       <c r="B7" s="17"/>
       <c r="AE7" s="16"/>
       <c r="AF7" s="16"/>
@@ -1708,7 +1703,7 @@
       <c r="AI7" s="16"/>
     </row>
     <row r="8" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="55"/>
+      <c r="A8" s="56"/>
       <c r="B8" s="17"/>
       <c r="AE8" s="16"/>
       <c r="AF8" s="16"/>
@@ -1718,7 +1713,7 @@
       <c r="AI8" s="16"/>
     </row>
     <row r="9" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="55"/>
+      <c r="A9" s="56"/>
       <c r="B9" s="17"/>
       <c r="AE9" s="16"/>
       <c r="AF9" s="16"/>
@@ -1728,7 +1723,7 @@
       <c r="AI9" s="16"/>
     </row>
     <row r="10" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="55"/>
+      <c r="A10" s="56"/>
       <c r="B10" s="17"/>
       <c r="AE10" s="16"/>
       <c r="AF10" s="16"/>
@@ -1738,7 +1733,7 @@
       <c r="AI10" s="16"/>
     </row>
     <row r="11" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="55"/>
+      <c r="A11" s="56"/>
       <c r="B11" s="17"/>
       <c r="AE11" s="16"/>
       <c r="AF11" s="16"/>
@@ -1748,7 +1743,7 @@
       <c r="AI11" s="16"/>
     </row>
     <row r="12" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="55"/>
+      <c r="A12" s="56"/>
       <c r="B12" s="17"/>
       <c r="AE12" s="16"/>
       <c r="AF12" s="16"/>
@@ -1758,7 +1753,7 @@
       <c r="AI12" s="16"/>
     </row>
     <row r="13" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="55"/>
+      <c r="A13" s="56"/>
       <c r="B13" s="17"/>
       <c r="AE13" s="16"/>
       <c r="AF13" s="16"/>
@@ -1768,7 +1763,7 @@
       <c r="AI13" s="16"/>
     </row>
     <row r="14" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="55"/>
+      <c r="A14" s="56"/>
       <c r="B14" s="17"/>
       <c r="AE14" s="16"/>
       <c r="AF14" s="16"/>
@@ -1778,710 +1773,710 @@
       <c r="AI14" s="16"/>
     </row>
     <row r="15" spans="1:35" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="55"/>
+      <c r="A15" s="56"/>
       <c r="B15" s="17"/>
       <c r="AE15" s="16"/>
       <c r="AF15" s="16"/>
-      <c r="AH15" s="50" t="s">
+      <c r="AH15" s="49" t="s">
         <v>64</v>
       </c>
-      <c r="AI15" s="52"/>
+      <c r="AI15" s="51"/>
     </row>
     <row r="16" spans="1:35" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="55"/>
+      <c r="A16" s="56"/>
       <c r="B16" s="17"/>
       <c r="AE16" s="16"/>
       <c r="AF16" s="16"/>
     </row>
     <row r="17" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55"/>
+      <c r="A17" s="56"/>
       <c r="B17" s="17"/>
       <c r="AE17" s="16"/>
       <c r="AF17" s="16"/>
     </row>
     <row r="18" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="55"/>
+      <c r="A18" s="56"/>
       <c r="B18" s="17"/>
       <c r="AE18" s="16"/>
       <c r="AF18" s="16"/>
     </row>
     <row r="19" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="55"/>
+      <c r="A19" s="56"/>
       <c r="B19" s="17"/>
       <c r="AE19" s="16"/>
       <c r="AF19" s="16"/>
     </row>
     <row r="20" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="55"/>
+      <c r="A20" s="56"/>
       <c r="B20" s="17"/>
       <c r="AE20" s="16"/>
       <c r="AF20" s="16"/>
     </row>
     <row r="21" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="55"/>
+      <c r="A21" s="56"/>
       <c r="B21" s="17"/>
       <c r="AE21" s="16"/>
       <c r="AF21" s="16"/>
     </row>
     <row r="22" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="55"/>
+      <c r="A22" s="56"/>
       <c r="B22" s="17"/>
       <c r="AE22" s="16"/>
       <c r="AF22" s="16"/>
     </row>
     <row r="23" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="55"/>
+      <c r="A23" s="56"/>
       <c r="B23" s="17"/>
       <c r="AE23" s="16"/>
       <c r="AF23" s="16"/>
     </row>
     <row r="24" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="55"/>
+      <c r="A24" s="56"/>
       <c r="B24" s="17"/>
       <c r="AE24" s="16"/>
       <c r="AF24" s="16"/>
     </row>
     <row r="25" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="55"/>
+      <c r="A25" s="56"/>
       <c r="B25" s="17"/>
       <c r="AE25" s="16"/>
       <c r="AF25" s="16"/>
     </row>
     <row r="26" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="55"/>
+      <c r="A26" s="56"/>
       <c r="B26" s="17"/>
       <c r="AE26" s="16"/>
       <c r="AF26" s="16"/>
     </row>
     <row r="27" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="55"/>
-      <c r="B27" s="56"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="57"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="57"/>
-      <c r="N27" s="57"/>
-      <c r="O27" s="57"/>
-      <c r="P27" s="57"/>
-      <c r="Q27" s="57"/>
-      <c r="R27" s="57"/>
-      <c r="S27" s="57"/>
-      <c r="T27" s="57"/>
-      <c r="U27" s="57"/>
-      <c r="V27" s="57"/>
-      <c r="W27" s="57"/>
-      <c r="X27" s="57"/>
-      <c r="Y27" s="57"/>
-      <c r="Z27" s="57"/>
-      <c r="AA27" s="57"/>
-      <c r="AB27" s="57"/>
-      <c r="AC27" s="57"/>
-      <c r="AD27" s="57"/>
-      <c r="AE27" s="68"/>
+      <c r="A27" s="56"/>
+      <c r="B27" s="57"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="58"/>
+      <c r="J27" s="58"/>
+      <c r="K27" s="58"/>
+      <c r="L27" s="58"/>
+      <c r="M27" s="58"/>
+      <c r="N27" s="58"/>
+      <c r="O27" s="58"/>
+      <c r="P27" s="58"/>
+      <c r="Q27" s="58"/>
+      <c r="R27" s="58"/>
+      <c r="S27" s="58"/>
+      <c r="T27" s="58"/>
+      <c r="U27" s="58"/>
+      <c r="V27" s="58"/>
+      <c r="W27" s="58"/>
+      <c r="X27" s="58"/>
+      <c r="Y27" s="58"/>
+      <c r="Z27" s="58"/>
+      <c r="AA27" s="58"/>
+      <c r="AB27" s="58"/>
+      <c r="AC27" s="58"/>
+      <c r="AD27" s="58"/>
+      <c r="AE27" s="69"/>
       <c r="AF27" s="16"/>
     </row>
     <row r="28" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="55"/>
-      <c r="B28" s="69"/>
-      <c r="C28" s="57"/>
-      <c r="D28" s="57"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="57"/>
-      <c r="K28" s="57"/>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="57"/>
-      <c r="O28" s="57"/>
-      <c r="P28" s="57"/>
-      <c r="Q28" s="57"/>
-      <c r="R28" s="57"/>
-      <c r="S28" s="57"/>
-      <c r="T28" s="57"/>
-      <c r="U28" s="57"/>
-      <c r="V28" s="57"/>
-      <c r="W28" s="57"/>
-      <c r="X28" s="57"/>
-      <c r="Y28" s="57"/>
-      <c r="Z28" s="57"/>
-      <c r="AA28" s="57"/>
-      <c r="AB28" s="57"/>
-      <c r="AC28" s="57"/>
-      <c r="AD28" s="57"/>
-      <c r="AE28" s="68"/>
+      <c r="A28" s="56"/>
+      <c r="B28" s="70"/>
+      <c r="C28" s="58"/>
+      <c r="D28" s="58"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="58"/>
+      <c r="L28" s="58"/>
+      <c r="M28" s="58"/>
+      <c r="N28" s="58"/>
+      <c r="O28" s="58"/>
+      <c r="P28" s="58"/>
+      <c r="Q28" s="58"/>
+      <c r="R28" s="58"/>
+      <c r="S28" s="58"/>
+      <c r="T28" s="58"/>
+      <c r="U28" s="58"/>
+      <c r="V28" s="58"/>
+      <c r="W28" s="58"/>
+      <c r="X28" s="58"/>
+      <c r="Y28" s="58"/>
+      <c r="Z28" s="58"/>
+      <c r="AA28" s="58"/>
+      <c r="AB28" s="58"/>
+      <c r="AC28" s="58"/>
+      <c r="AD28" s="58"/>
+      <c r="AE28" s="69"/>
       <c r="AF28" s="16"/>
     </row>
     <row r="29" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="55"/>
-      <c r="B29" s="58" t="str">
+      <c r="A29" s="56"/>
+      <c r="B29" s="59" t="str">
         <f>H40</f>
         <v>00-01-00</v>
       </c>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="60">
-        <f>AE44</f>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61" t="str">
+        <f>UPPER(AE44)</f>
         <v>0</v>
       </c>
-      <c r="G29" s="60"/>
-      <c r="H29" s="60"/>
-      <c r="I29" s="60" t="s">
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="J29" s="60"/>
-      <c r="K29" s="60"/>
-      <c r="L29" s="60"/>
-      <c r="M29" s="60"/>
-      <c r="N29" s="60"/>
-      <c r="O29" s="60"/>
-      <c r="P29" s="60"/>
-      <c r="Q29" s="60"/>
-      <c r="R29" s="60"/>
-      <c r="S29" s="60"/>
-      <c r="T29" s="60"/>
-      <c r="U29" s="60"/>
-      <c r="V29" s="60"/>
-      <c r="W29" s="60"/>
-      <c r="X29" s="60"/>
-      <c r="Y29" s="60"/>
-      <c r="Z29" s="61"/>
-      <c r="AA29" s="62"/>
-      <c r="AB29" s="61"/>
-      <c r="AC29" s="62"/>
-      <c r="AD29" s="61"/>
-      <c r="AE29" s="70"/>
+      <c r="J29" s="61"/>
+      <c r="K29" s="61"/>
+      <c r="L29" s="61"/>
+      <c r="M29" s="61"/>
+      <c r="N29" s="61"/>
+      <c r="O29" s="61"/>
+      <c r="P29" s="61"/>
+      <c r="Q29" s="61"/>
+      <c r="R29" s="61"/>
+      <c r="S29" s="61"/>
+      <c r="T29" s="61"/>
+      <c r="U29" s="61"/>
+      <c r="V29" s="61"/>
+      <c r="W29" s="61"/>
+      <c r="X29" s="61"/>
+      <c r="Y29" s="61"/>
+      <c r="Z29" s="62"/>
+      <c r="AA29" s="63"/>
+      <c r="AB29" s="62"/>
+      <c r="AC29" s="63"/>
+      <c r="AD29" s="62"/>
+      <c r="AE29" s="71"/>
       <c r="AF29" s="16"/>
     </row>
     <row r="30" spans="1:32" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="55"/>
-      <c r="B30" s="58"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="60"/>
-      <c r="J30" s="60"/>
-      <c r="K30" s="60"/>
-      <c r="L30" s="60"/>
-      <c r="M30" s="60"/>
-      <c r="N30" s="60"/>
-      <c r="O30" s="60"/>
-      <c r="P30" s="60"/>
-      <c r="Q30" s="60"/>
-      <c r="R30" s="60"/>
-      <c r="S30" s="60"/>
-      <c r="T30" s="60"/>
-      <c r="U30" s="60"/>
-      <c r="V30" s="60"/>
-      <c r="W30" s="60"/>
-      <c r="X30" s="60"/>
-      <c r="Y30" s="60"/>
-      <c r="Z30" s="71">
+      <c r="A30" s="56"/>
+      <c r="B30" s="59"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="61"/>
+      <c r="G30" s="61"/>
+      <c r="H30" s="61"/>
+      <c r="I30" s="61"/>
+      <c r="J30" s="61"/>
+      <c r="K30" s="61"/>
+      <c r="L30" s="61"/>
+      <c r="M30" s="61"/>
+      <c r="N30" s="61"/>
+      <c r="O30" s="61"/>
+      <c r="P30" s="61"/>
+      <c r="Q30" s="61"/>
+      <c r="R30" s="61"/>
+      <c r="S30" s="61"/>
+      <c r="T30" s="61"/>
+      <c r="U30" s="61"/>
+      <c r="V30" s="61"/>
+      <c r="W30" s="61"/>
+      <c r="X30" s="61"/>
+      <c r="Y30" s="61"/>
+      <c r="Z30" s="72">
         <f>AI7</f>
         <v>0</v>
       </c>
-      <c r="AA30" s="60"/>
-      <c r="AB30" s="71">
+      <c r="AA30" s="61"/>
+      <c r="AB30" s="72">
         <f>AI8</f>
         <v>0</v>
       </c>
-      <c r="AC30" s="60"/>
-      <c r="AD30" s="71">
+      <c r="AC30" s="61"/>
+      <c r="AD30" s="72">
         <f>AI9</f>
         <v>0</v>
       </c>
-      <c r="AE30" s="67"/>
+      <c r="AE30" s="68"/>
       <c r="AF30" s="16"/>
     </row>
     <row r="31" spans="1:32" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="55"/>
-      <c r="B31" s="80" t="s">
+      <c r="A31" s="56"/>
+      <c r="B31" s="81" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="81"/>
-      <c r="D31" s="81"/>
-      <c r="E31" s="81"/>
-      <c r="F31" s="81" t="s">
+      <c r="C31" s="82"/>
+      <c r="D31" s="82"/>
+      <c r="E31" s="82"/>
+      <c r="F31" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="G31" s="81"/>
-      <c r="H31" s="81"/>
-      <c r="I31" s="81" t="s">
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="J31" s="81"/>
-      <c r="K31" s="81"/>
-      <c r="L31" s="81"/>
-      <c r="M31" s="81"/>
-      <c r="N31" s="81"/>
-      <c r="O31" s="81"/>
-      <c r="P31" s="81"/>
-      <c r="Q31" s="81"/>
-      <c r="R31" s="81"/>
-      <c r="S31" s="81"/>
-      <c r="T31" s="81"/>
-      <c r="U31" s="81"/>
-      <c r="V31" s="81"/>
-      <c r="W31" s="81"/>
-      <c r="X31" s="81"/>
-      <c r="Y31" s="81"/>
-      <c r="Z31" s="72" t="s">
+      <c r="J31" s="82"/>
+      <c r="K31" s="82"/>
+      <c r="L31" s="82"/>
+      <c r="M31" s="82"/>
+      <c r="N31" s="82"/>
+      <c r="O31" s="82"/>
+      <c r="P31" s="82"/>
+      <c r="Q31" s="82"/>
+      <c r="R31" s="82"/>
+      <c r="S31" s="82"/>
+      <c r="T31" s="82"/>
+      <c r="U31" s="82"/>
+      <c r="V31" s="82"/>
+      <c r="W31" s="82"/>
+      <c r="X31" s="82"/>
+      <c r="Y31" s="82"/>
+      <c r="Z31" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="AA31" s="72"/>
-      <c r="AB31" s="72" t="s">
+      <c r="AA31" s="73"/>
+      <c r="AB31" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="AC31" s="72"/>
-      <c r="AD31" s="72" t="s">
+      <c r="AC31" s="73"/>
+      <c r="AD31" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="AE31" s="73"/>
+      <c r="AE31" s="74"/>
       <c r="AF31" s="16"/>
     </row>
     <row r="32" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="55"/>
-      <c r="B32" s="74"/>
-      <c r="C32" s="75"/>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
-      <c r="I32" s="75"/>
-      <c r="J32" s="75"/>
-      <c r="K32" s="75"/>
-      <c r="L32" s="75"/>
-      <c r="M32" s="75"/>
-      <c r="N32" s="75"/>
-      <c r="O32" s="75"/>
-      <c r="P32" s="75"/>
-      <c r="Q32" s="75"/>
-      <c r="R32" s="75"/>
-      <c r="S32" s="75"/>
-      <c r="T32" s="75"/>
-      <c r="U32" s="75"/>
-      <c r="V32" s="75"/>
-      <c r="W32" s="75"/>
-      <c r="X32" s="75"/>
-      <c r="Y32" s="75"/>
-      <c r="Z32" s="75"/>
-      <c r="AA32" s="75"/>
-      <c r="AB32" s="75"/>
-      <c r="AC32" s="75"/>
-      <c r="AD32" s="75"/>
-      <c r="AE32" s="76"/>
+      <c r="A32" s="56"/>
+      <c r="B32" s="75"/>
+      <c r="C32" s="76"/>
+      <c r="D32" s="76"/>
+      <c r="E32" s="76"/>
+      <c r="F32" s="76"/>
+      <c r="G32" s="76"/>
+      <c r="H32" s="76"/>
+      <c r="I32" s="76"/>
+      <c r="J32" s="76"/>
+      <c r="K32" s="76"/>
+      <c r="L32" s="76"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="76"/>
+      <c r="O32" s="76"/>
+      <c r="P32" s="76"/>
+      <c r="Q32" s="76"/>
+      <c r="R32" s="76"/>
+      <c r="S32" s="76"/>
+      <c r="T32" s="76"/>
+      <c r="U32" s="76"/>
+      <c r="V32" s="76"/>
+      <c r="W32" s="76"/>
+      <c r="X32" s="76"/>
+      <c r="Y32" s="76"/>
+      <c r="Z32" s="76"/>
+      <c r="AA32" s="76"/>
+      <c r="AB32" s="76"/>
+      <c r="AC32" s="76"/>
+      <c r="AD32" s="76"/>
+      <c r="AE32" s="77"/>
       <c r="AF32" s="16"/>
     </row>
     <row r="33" spans="1:32" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="55"/>
-      <c r="B33" s="77"/>
-      <c r="C33" s="78"/>
-      <c r="D33" s="78"/>
-      <c r="E33" s="78"/>
-      <c r="F33" s="78"/>
-      <c r="G33" s="78"/>
-      <c r="H33" s="78"/>
-      <c r="I33" s="78"/>
-      <c r="J33" s="78"/>
-      <c r="K33" s="78"/>
-      <c r="L33" s="78"/>
-      <c r="M33" s="78"/>
-      <c r="N33" s="78"/>
-      <c r="O33" s="78"/>
-      <c r="P33" s="78"/>
-      <c r="Q33" s="78"/>
-      <c r="R33" s="78"/>
-      <c r="S33" s="78"/>
-      <c r="T33" s="78"/>
-      <c r="U33" s="78"/>
-      <c r="V33" s="78"/>
-      <c r="W33" s="78"/>
-      <c r="X33" s="78"/>
-      <c r="Y33" s="78"/>
-      <c r="Z33" s="78"/>
-      <c r="AA33" s="78"/>
-      <c r="AB33" s="78"/>
-      <c r="AC33" s="78"/>
-      <c r="AD33" s="78"/>
-      <c r="AE33" s="79"/>
+      <c r="A33" s="56"/>
+      <c r="B33" s="78"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="79"/>
+      <c r="G33" s="79"/>
+      <c r="H33" s="79"/>
+      <c r="I33" s="79"/>
+      <c r="J33" s="79"/>
+      <c r="K33" s="79"/>
+      <c r="L33" s="79"/>
+      <c r="M33" s="79"/>
+      <c r="N33" s="79"/>
+      <c r="O33" s="79"/>
+      <c r="P33" s="79"/>
+      <c r="Q33" s="79"/>
+      <c r="R33" s="79"/>
+      <c r="S33" s="79"/>
+      <c r="T33" s="79"/>
+      <c r="U33" s="79"/>
+      <c r="V33" s="79"/>
+      <c r="W33" s="79"/>
+      <c r="X33" s="79"/>
+      <c r="Y33" s="79"/>
+      <c r="Z33" s="79"/>
+      <c r="AA33" s="79"/>
+      <c r="AB33" s="79"/>
+      <c r="AC33" s="79"/>
+      <c r="AD33" s="79"/>
+      <c r="AE33" s="80"/>
       <c r="AF33" s="16"/>
     </row>
     <row r="34" spans="1:32" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="55"/>
-      <c r="B34" s="63" t="s">
+      <c r="A34" s="56"/>
+      <c r="B34" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="C34" s="64"/>
-      <c r="D34" s="64"/>
-      <c r="E34" s="64"/>
-      <c r="F34" s="65">
-        <f>AI12</f>
-        <v>0</v>
-      </c>
-      <c r="G34" s="65"/>
-      <c r="H34" s="65"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="65"/>
-      <c r="K34" s="65"/>
-      <c r="L34" s="65"/>
-      <c r="M34" s="65"/>
-      <c r="N34" s="65"/>
-      <c r="O34" s="65"/>
-      <c r="P34" s="65"/>
-      <c r="Q34" s="65"/>
-      <c r="R34" s="65"/>
-      <c r="S34" s="65"/>
-      <c r="T34" s="65"/>
-      <c r="U34" s="65"/>
-      <c r="V34" s="65"/>
-      <c r="W34" s="65"/>
-      <c r="X34" s="65"/>
-      <c r="Y34" s="65"/>
-      <c r="Z34" s="65"/>
-      <c r="AA34" s="65"/>
-      <c r="AB34" s="65"/>
-      <c r="AC34" s="65"/>
-      <c r="AD34" s="65"/>
-      <c r="AE34" s="66"/>
+      <c r="C34" s="65"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="66" t="str">
+        <f>UPPER(AI12)</f>
+        <v/>
+      </c>
+      <c r="G34" s="66"/>
+      <c r="H34" s="66"/>
+      <c r="I34" s="66"/>
+      <c r="J34" s="66"/>
+      <c r="K34" s="66"/>
+      <c r="L34" s="66"/>
+      <c r="M34" s="66"/>
+      <c r="N34" s="66"/>
+      <c r="O34" s="66"/>
+      <c r="P34" s="66"/>
+      <c r="Q34" s="66"/>
+      <c r="R34" s="66"/>
+      <c r="S34" s="66"/>
+      <c r="T34" s="66"/>
+      <c r="U34" s="66"/>
+      <c r="V34" s="66"/>
+      <c r="W34" s="66"/>
+      <c r="X34" s="66"/>
+      <c r="Y34" s="66"/>
+      <c r="Z34" s="66"/>
+      <c r="AA34" s="66"/>
+      <c r="AB34" s="66"/>
+      <c r="AC34" s="66"/>
+      <c r="AD34" s="66"/>
+      <c r="AE34" s="67"/>
       <c r="AF34" s="16"/>
     </row>
     <row r="35" spans="1:32" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="55"/>
-      <c r="B35" s="63" t="s">
+      <c r="A35" s="56"/>
+      <c r="B35" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="64"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="64"/>
-      <c r="F35" s="65">
-        <f>AI13</f>
-        <v>0</v>
-      </c>
-      <c r="G35" s="65"/>
-      <c r="H35" s="65"/>
-      <c r="I35" s="65"/>
-      <c r="J35" s="65"/>
-      <c r="K35" s="65"/>
-      <c r="L35" s="65"/>
-      <c r="M35" s="65"/>
-      <c r="N35" s="65"/>
-      <c r="O35" s="65"/>
-      <c r="P35" s="65"/>
-      <c r="Q35" s="65"/>
-      <c r="R35" s="65"/>
-      <c r="S35" s="65"/>
-      <c r="T35" s="65"/>
-      <c r="U35" s="65"/>
-      <c r="V35" s="65"/>
-      <c r="W35" s="65"/>
-      <c r="X35" s="65"/>
-      <c r="Y35" s="65"/>
-      <c r="Z35" s="65"/>
-      <c r="AA35" s="65"/>
-      <c r="AB35" s="65"/>
-      <c r="AC35" s="65"/>
-      <c r="AD35" s="65"/>
-      <c r="AE35" s="66"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="66" t="str">
+        <f>UPPER(AI13)</f>
+        <v/>
+      </c>
+      <c r="G35" s="66"/>
+      <c r="H35" s="66"/>
+      <c r="I35" s="66"/>
+      <c r="J35" s="66"/>
+      <c r="K35" s="66"/>
+      <c r="L35" s="66"/>
+      <c r="M35" s="66"/>
+      <c r="N35" s="66"/>
+      <c r="O35" s="66"/>
+      <c r="P35" s="66"/>
+      <c r="Q35" s="66"/>
+      <c r="R35" s="66"/>
+      <c r="S35" s="66"/>
+      <c r="T35" s="66"/>
+      <c r="U35" s="66"/>
+      <c r="V35" s="66"/>
+      <c r="W35" s="66"/>
+      <c r="X35" s="66"/>
+      <c r="Y35" s="66"/>
+      <c r="Z35" s="66"/>
+      <c r="AA35" s="66"/>
+      <c r="AB35" s="66"/>
+      <c r="AC35" s="66"/>
+      <c r="AD35" s="66"/>
+      <c r="AE35" s="67"/>
       <c r="AF35" s="16"/>
     </row>
     <row r="36" spans="1:32" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="55"/>
-      <c r="B36" s="63" t="s">
+      <c r="A36" s="56"/>
+      <c r="B36" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="64"/>
-      <c r="D36" s="64"/>
-      <c r="E36" s="64"/>
-      <c r="F36" s="65">
-        <f>AI11</f>
-        <v>0</v>
-      </c>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
-      <c r="I36" s="65"/>
-      <c r="J36" s="65"/>
-      <c r="K36" s="65"/>
-      <c r="L36" s="65"/>
-      <c r="M36" s="65"/>
-      <c r="N36" s="65"/>
-      <c r="O36" s="65"/>
-      <c r="P36" s="65"/>
-      <c r="Q36" s="65"/>
-      <c r="R36" s="65"/>
-      <c r="S36" s="65"/>
-      <c r="T36" s="65"/>
-      <c r="U36" s="65"/>
-      <c r="V36" s="65"/>
-      <c r="W36" s="65"/>
-      <c r="X36" s="65"/>
-      <c r="Y36" s="65"/>
-      <c r="Z36" s="65"/>
-      <c r="AA36" s="65"/>
-      <c r="AB36" s="65"/>
-      <c r="AC36" s="65"/>
-      <c r="AD36" s="65"/>
-      <c r="AE36" s="66"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="66" t="str">
+        <f>UPPER(AI11)</f>
+        <v/>
+      </c>
+      <c r="G36" s="66"/>
+      <c r="H36" s="66"/>
+      <c r="I36" s="66"/>
+      <c r="J36" s="66"/>
+      <c r="K36" s="66"/>
+      <c r="L36" s="66"/>
+      <c r="M36" s="66"/>
+      <c r="N36" s="66"/>
+      <c r="O36" s="66"/>
+      <c r="P36" s="66"/>
+      <c r="Q36" s="66"/>
+      <c r="R36" s="66"/>
+      <c r="S36" s="66"/>
+      <c r="T36" s="66"/>
+      <c r="U36" s="66"/>
+      <c r="V36" s="66"/>
+      <c r="W36" s="66"/>
+      <c r="X36" s="66"/>
+      <c r="Y36" s="66"/>
+      <c r="Z36" s="66"/>
+      <c r="AA36" s="66"/>
+      <c r="AB36" s="66"/>
+      <c r="AC36" s="66"/>
+      <c r="AD36" s="66"/>
+      <c r="AE36" s="67"/>
       <c r="AF36" s="16"/>
     </row>
     <row r="37" spans="1:32" ht="56.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="55"/>
-      <c r="B37" s="63" t="s">
+      <c r="A37" s="56"/>
+      <c r="B37" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="C37" s="64"/>
-      <c r="D37" s="64"/>
-      <c r="E37" s="64"/>
-      <c r="F37" s="60" t="s">
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="G37" s="60"/>
-      <c r="H37" s="60"/>
-      <c r="I37" s="60"/>
-      <c r="J37" s="60"/>
-      <c r="K37" s="60"/>
-      <c r="L37" s="60"/>
-      <c r="M37" s="60"/>
-      <c r="N37" s="60"/>
-      <c r="O37" s="60"/>
-      <c r="P37" s="60"/>
-      <c r="Q37" s="60"/>
-      <c r="R37" s="60"/>
-      <c r="S37" s="60"/>
-      <c r="T37" s="60"/>
-      <c r="U37" s="60"/>
-      <c r="V37" s="60"/>
-      <c r="W37" s="60"/>
-      <c r="X37" s="60"/>
-      <c r="Y37" s="60"/>
-      <c r="Z37" s="60"/>
-      <c r="AA37" s="60"/>
-      <c r="AB37" s="60"/>
-      <c r="AC37" s="60"/>
-      <c r="AD37" s="60"/>
-      <c r="AE37" s="67"/>
+      <c r="G37" s="61"/>
+      <c r="H37" s="61"/>
+      <c r="I37" s="61"/>
+      <c r="J37" s="61"/>
+      <c r="K37" s="61"/>
+      <c r="L37" s="61"/>
+      <c r="M37" s="61"/>
+      <c r="N37" s="61"/>
+      <c r="O37" s="61"/>
+      <c r="P37" s="61"/>
+      <c r="Q37" s="61"/>
+      <c r="R37" s="61"/>
+      <c r="S37" s="61"/>
+      <c r="T37" s="61"/>
+      <c r="U37" s="61"/>
+      <c r="V37" s="61"/>
+      <c r="W37" s="61"/>
+      <c r="X37" s="61"/>
+      <c r="Y37" s="61"/>
+      <c r="Z37" s="61"/>
+      <c r="AA37" s="61"/>
+      <c r="AB37" s="61"/>
+      <c r="AC37" s="61"/>
+      <c r="AD37" s="61"/>
+      <c r="AE37" s="68"/>
       <c r="AF37" s="16"/>
     </row>
     <row r="38" spans="1:32" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="18"/>
-      <c r="B38" s="80" t="s">
+      <c r="B38" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="81"/>
-      <c r="D38" s="82" t="s">
+      <c r="C38" s="82"/>
+      <c r="D38" s="83" t="s">
         <v>37</v>
       </c>
-      <c r="E38" s="82"/>
-      <c r="F38" s="82"/>
-      <c r="G38" s="82"/>
-      <c r="H38" s="82"/>
-      <c r="I38" s="82"/>
-      <c r="J38" s="83" t="s">
+      <c r="E38" s="83"/>
+      <c r="F38" s="83"/>
+      <c r="G38" s="83"/>
+      <c r="H38" s="83"/>
+      <c r="I38" s="83"/>
+      <c r="J38" s="84" t="s">
         <v>38</v>
       </c>
-      <c r="K38" s="83"/>
-      <c r="L38" s="83"/>
-      <c r="M38" s="83"/>
-      <c r="N38" s="83"/>
-      <c r="O38" s="83"/>
-      <c r="P38" s="83"/>
-      <c r="Q38" s="83"/>
-      <c r="R38" s="83"/>
-      <c r="S38" s="83"/>
-      <c r="T38" s="83"/>
-      <c r="U38" s="83"/>
-      <c r="V38" s="83"/>
-      <c r="W38" s="83"/>
-      <c r="X38" s="83"/>
-      <c r="Y38" s="83"/>
-      <c r="Z38" s="83"/>
-      <c r="AA38" s="83"/>
-      <c r="AB38" s="83"/>
-      <c r="AC38" s="83"/>
-      <c r="AD38" s="83"/>
-      <c r="AE38" s="84"/>
+      <c r="K38" s="84"/>
+      <c r="L38" s="84"/>
+      <c r="M38" s="84"/>
+      <c r="N38" s="84"/>
+      <c r="O38" s="84"/>
+      <c r="P38" s="84"/>
+      <c r="Q38" s="84"/>
+      <c r="R38" s="84"/>
+      <c r="S38" s="84"/>
+      <c r="T38" s="84"/>
+      <c r="U38" s="84"/>
+      <c r="V38" s="84"/>
+      <c r="W38" s="84"/>
+      <c r="X38" s="84"/>
+      <c r="Y38" s="84"/>
+      <c r="Z38" s="84"/>
+      <c r="AA38" s="84"/>
+      <c r="AB38" s="84"/>
+      <c r="AC38" s="84"/>
+      <c r="AD38" s="84"/>
+      <c r="AE38" s="85"/>
       <c r="AF38" s="16"/>
     </row>
     <row r="39" spans="1:32" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="18"/>
-      <c r="B39" s="87"/>
-      <c r="C39" s="60"/>
-      <c r="D39" s="81" t="s">
+      <c r="B39" s="88"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="E39" s="81"/>
-      <c r="F39" s="81" t="s">
+      <c r="E39" s="82"/>
+      <c r="F39" s="82" t="s">
         <v>40</v>
       </c>
-      <c r="G39" s="81"/>
-      <c r="H39" s="81" t="s">
+      <c r="G39" s="82"/>
+      <c r="H39" s="82" t="s">
         <v>25</v>
       </c>
-      <c r="I39" s="81"/>
-      <c r="J39" s="92" t="str">
-        <f>"INSTRUMENT LIST FOR "&amp;AI15</f>
+      <c r="I39" s="82"/>
+      <c r="J39" s="93" t="str">
+        <f>"INSTRUMENT LIST FOR "&amp;UPPER(AI15)</f>
         <v xml:space="preserve">INSTRUMENT LIST FOR </v>
       </c>
-      <c r="K39" s="92"/>
-      <c r="L39" s="92"/>
-      <c r="M39" s="92"/>
-      <c r="N39" s="92"/>
-      <c r="O39" s="92"/>
-      <c r="P39" s="92"/>
-      <c r="Q39" s="92"/>
-      <c r="R39" s="92"/>
-      <c r="S39" s="92"/>
-      <c r="T39" s="92"/>
-      <c r="U39" s="92"/>
-      <c r="V39" s="92"/>
-      <c r="W39" s="92"/>
-      <c r="X39" s="92"/>
-      <c r="Y39" s="92"/>
-      <c r="Z39" s="92"/>
-      <c r="AA39" s="92"/>
-      <c r="AB39" s="92"/>
-      <c r="AC39" s="92"/>
-      <c r="AD39" s="92"/>
-      <c r="AE39" s="93"/>
+      <c r="K39" s="93"/>
+      <c r="L39" s="93"/>
+      <c r="M39" s="93"/>
+      <c r="N39" s="93"/>
+      <c r="O39" s="93"/>
+      <c r="P39" s="93"/>
+      <c r="Q39" s="93"/>
+      <c r="R39" s="93"/>
+      <c r="S39" s="93"/>
+      <c r="T39" s="93"/>
+      <c r="U39" s="93"/>
+      <c r="V39" s="93"/>
+      <c r="W39" s="93"/>
+      <c r="X39" s="93"/>
+      <c r="Y39" s="93"/>
+      <c r="Z39" s="93"/>
+      <c r="AA39" s="93"/>
+      <c r="AB39" s="93"/>
+      <c r="AC39" s="93"/>
+      <c r="AD39" s="93"/>
+      <c r="AE39" s="94"/>
       <c r="AF39" s="16"/>
     </row>
     <row r="40" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="18"/>
-      <c r="B40" s="80" t="s">
+      <c r="B40" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="81"/>
-      <c r="D40" s="60">
+      <c r="C40" s="82"/>
+      <c r="D40" s="61">
         <f>Z30</f>
         <v>0</v>
       </c>
-      <c r="E40" s="60"/>
-      <c r="F40" s="85"/>
-      <c r="G40" s="88"/>
-      <c r="H40" s="86" t="str">
+      <c r="E40" s="61"/>
+      <c r="F40" s="86"/>
+      <c r="G40" s="89"/>
+      <c r="H40" s="87" t="str">
         <f>TEXT(AI6,"DD-MM-YY")</f>
         <v>00-01-00</v>
       </c>
-      <c r="I40" s="86"/>
-      <c r="J40" s="92"/>
-      <c r="K40" s="92"/>
-      <c r="L40" s="92"/>
-      <c r="M40" s="92"/>
-      <c r="N40" s="92"/>
-      <c r="O40" s="92"/>
-      <c r="P40" s="92"/>
-      <c r="Q40" s="92"/>
-      <c r="R40" s="92"/>
-      <c r="S40" s="92"/>
-      <c r="T40" s="92"/>
-      <c r="U40" s="92"/>
-      <c r="V40" s="92"/>
-      <c r="W40" s="92"/>
-      <c r="X40" s="92"/>
-      <c r="Y40" s="92"/>
-      <c r="Z40" s="92"/>
-      <c r="AA40" s="92"/>
-      <c r="AB40" s="92"/>
-      <c r="AC40" s="92"/>
-      <c r="AD40" s="92"/>
-      <c r="AE40" s="93"/>
+      <c r="I40" s="87"/>
+      <c r="J40" s="93"/>
+      <c r="K40" s="93"/>
+      <c r="L40" s="93"/>
+      <c r="M40" s="93"/>
+      <c r="N40" s="93"/>
+      <c r="O40" s="93"/>
+      <c r="P40" s="93"/>
+      <c r="Q40" s="93"/>
+      <c r="R40" s="93"/>
+      <c r="S40" s="93"/>
+      <c r="T40" s="93"/>
+      <c r="U40" s="93"/>
+      <c r="V40" s="93"/>
+      <c r="W40" s="93"/>
+      <c r="X40" s="93"/>
+      <c r="Y40" s="93"/>
+      <c r="Z40" s="93"/>
+      <c r="AA40" s="93"/>
+      <c r="AB40" s="93"/>
+      <c r="AC40" s="93"/>
+      <c r="AD40" s="93"/>
+      <c r="AE40" s="94"/>
       <c r="AF40" s="16"/>
     </row>
     <row r="41" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="18"/>
-      <c r="B41" s="80" t="s">
+      <c r="B41" s="81" t="s">
         <v>42</v>
       </c>
-      <c r="C41" s="81"/>
-      <c r="D41" s="60">
+      <c r="C41" s="82"/>
+      <c r="D41" s="61">
         <f>AB30</f>
         <v>0</v>
       </c>
-      <c r="E41" s="60"/>
-      <c r="F41" s="85"/>
-      <c r="G41" s="88"/>
-      <c r="H41" s="86" t="e">
+      <c r="E41" s="61"/>
+      <c r="F41" s="86"/>
+      <c r="G41" s="89"/>
+      <c r="H41" s="87" t="e">
         <f>H40+1</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I41" s="86"/>
-      <c r="J41" s="92"/>
-      <c r="K41" s="92"/>
-      <c r="L41" s="92"/>
-      <c r="M41" s="92"/>
-      <c r="N41" s="92"/>
-      <c r="O41" s="92"/>
-      <c r="P41" s="92"/>
-      <c r="Q41" s="92"/>
-      <c r="R41" s="92"/>
-      <c r="S41" s="92"/>
-      <c r="T41" s="92"/>
-      <c r="U41" s="92"/>
-      <c r="V41" s="92"/>
-      <c r="W41" s="92"/>
-      <c r="X41" s="92"/>
-      <c r="Y41" s="92"/>
-      <c r="Z41" s="92"/>
-      <c r="AA41" s="92"/>
-      <c r="AB41" s="92"/>
-      <c r="AC41" s="92"/>
-      <c r="AD41" s="92"/>
-      <c r="AE41" s="93"/>
+      <c r="I41" s="87"/>
+      <c r="J41" s="93"/>
+      <c r="K41" s="93"/>
+      <c r="L41" s="93"/>
+      <c r="M41" s="93"/>
+      <c r="N41" s="93"/>
+      <c r="O41" s="93"/>
+      <c r="P41" s="93"/>
+      <c r="Q41" s="93"/>
+      <c r="R41" s="93"/>
+      <c r="S41" s="93"/>
+      <c r="T41" s="93"/>
+      <c r="U41" s="93"/>
+      <c r="V41" s="93"/>
+      <c r="W41" s="93"/>
+      <c r="X41" s="93"/>
+      <c r="Y41" s="93"/>
+      <c r="Z41" s="93"/>
+      <c r="AA41" s="93"/>
+      <c r="AB41" s="93"/>
+      <c r="AC41" s="93"/>
+      <c r="AD41" s="93"/>
+      <c r="AE41" s="94"/>
       <c r="AF41" s="16"/>
     </row>
     <row r="42" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="18"/>
-      <c r="B42" s="80" t="s">
+      <c r="B42" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="C42" s="81"/>
-      <c r="D42" s="60">
+      <c r="C42" s="82"/>
+      <c r="D42" s="61">
         <f>AD30</f>
         <v>0</v>
       </c>
-      <c r="E42" s="60"/>
-      <c r="F42" s="85"/>
-      <c r="G42" s="85"/>
-      <c r="H42" s="86" t="e">
+      <c r="E42" s="61"/>
+      <c r="F42" s="86"/>
+      <c r="G42" s="86"/>
+      <c r="H42" s="87" t="e">
         <f>H41</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I42" s="86"/>
-      <c r="J42" s="92"/>
-      <c r="K42" s="92"/>
-      <c r="L42" s="92"/>
-      <c r="M42" s="92"/>
-      <c r="N42" s="92"/>
-      <c r="O42" s="92"/>
-      <c r="P42" s="92"/>
-      <c r="Q42" s="92"/>
-      <c r="R42" s="92"/>
-      <c r="S42" s="92"/>
-      <c r="T42" s="92"/>
-      <c r="U42" s="92"/>
-      <c r="V42" s="92"/>
-      <c r="W42" s="92"/>
-      <c r="X42" s="92"/>
-      <c r="Y42" s="92"/>
-      <c r="Z42" s="92"/>
-      <c r="AA42" s="92"/>
-      <c r="AB42" s="92"/>
-      <c r="AC42" s="92"/>
-      <c r="AD42" s="92"/>
-      <c r="AE42" s="93"/>
+      <c r="I42" s="87"/>
+      <c r="J42" s="93"/>
+      <c r="K42" s="93"/>
+      <c r="L42" s="93"/>
+      <c r="M42" s="93"/>
+      <c r="N42" s="93"/>
+      <c r="O42" s="93"/>
+      <c r="P42" s="93"/>
+      <c r="Q42" s="93"/>
+      <c r="R42" s="93"/>
+      <c r="S42" s="93"/>
+      <c r="T42" s="93"/>
+      <c r="U42" s="93"/>
+      <c r="V42" s="93"/>
+      <c r="W42" s="93"/>
+      <c r="X42" s="93"/>
+      <c r="Y42" s="93"/>
+      <c r="Z42" s="93"/>
+      <c r="AA42" s="93"/>
+      <c r="AB42" s="93"/>
+      <c r="AC42" s="93"/>
+      <c r="AD42" s="93"/>
+      <c r="AE42" s="94"/>
       <c r="AF42" s="16"/>
     </row>
     <row r="43" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2495,14 +2490,14 @@
       <c r="H43" s="20"/>
       <c r="I43" s="20"/>
       <c r="AA43" s="21"/>
-      <c r="AB43" s="89" t="s">
+      <c r="AB43" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="AC43" s="90"/>
-      <c r="AD43" s="89" t="s">
+      <c r="AC43" s="91"/>
+      <c r="AD43" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="AE43" s="91"/>
+      <c r="AE43" s="92"/>
       <c r="AF43" s="16"/>
     </row>
     <row r="44" spans="1:32" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2654,47 +2649,39 @@
       <c r="D48" s="39"/>
       <c r="E48" s="39"/>
       <c r="F48" s="25"/>
-      <c r="G48" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="H48" s="41" t="s">
+      <c r="G48" s="53"/>
+      <c r="H48" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="I48" s="42"/>
-      <c r="J48" s="42"/>
-      <c r="K48" s="42"/>
-      <c r="L48" s="43"/>
-      <c r="M48" s="44"/>
-      <c r="N48" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="O48" s="41" t="s">
+      <c r="I48" s="41"/>
+      <c r="J48" s="41"/>
+      <c r="K48" s="41"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="43"/>
+      <c r="N48" s="53"/>
+      <c r="O48" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="P48" s="43"/>
+      <c r="P48" s="42"/>
       <c r="Q48" s="25"/>
-      <c r="R48" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="S48" s="41" t="s">
+      <c r="R48" s="53"/>
+      <c r="S48" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="T48" s="42"/>
-      <c r="U48" s="43"/>
-      <c r="V48" s="44"/>
-      <c r="W48" s="40" t="b">
-        <v>1</v>
-      </c>
-      <c r="X48" s="41" t="s">
+      <c r="T48" s="41"/>
+      <c r="U48" s="42"/>
+      <c r="V48" s="43"/>
+      <c r="W48" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="X48" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="Y48" s="42"/>
-      <c r="Z48" s="43"/>
+      <c r="Y48" s="41"/>
+      <c r="Z48" s="42"/>
       <c r="AA48" s="25"/>
-      <c r="AB48" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC48" s="41" t="s">
+      <c r="AB48" s="53"/>
+      <c r="AC48" s="40" t="s">
         <v>53</v>
       </c>
       <c r="AE48" s="16"/>
@@ -2702,105 +2689,105 @@
     </row>
     <row r="49" spans="1:32" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="18"/>
-      <c r="B49" s="45"/>
+      <c r="B49" s="44"/>
       <c r="C49" s="39"/>
       <c r="D49" s="39"/>
       <c r="E49" s="39"/>
-      <c r="F49" s="46"/>
-      <c r="G49" s="47"/>
-      <c r="H49" s="47"/>
-      <c r="I49" s="47"/>
-      <c r="J49" s="47"/>
-      <c r="K49" s="47"/>
-      <c r="L49" s="48"/>
-      <c r="M49" s="46"/>
-      <c r="N49" s="47"/>
-      <c r="O49" s="47"/>
-      <c r="P49" s="48"/>
-      <c r="Q49" s="46"/>
-      <c r="R49" s="47"/>
-      <c r="S49" s="47"/>
-      <c r="T49" s="47"/>
-      <c r="U49" s="48"/>
-      <c r="V49" s="46"/>
-      <c r="W49" s="47"/>
-      <c r="X49" s="47"/>
-      <c r="Y49" s="47"/>
-      <c r="Z49" s="48"/>
-      <c r="AA49" s="46"/>
-      <c r="AB49" s="47"/>
-      <c r="AC49" s="47"/>
-      <c r="AD49" s="47"/>
-      <c r="AE49" s="49"/>
+      <c r="F49" s="45"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="46"/>
+      <c r="I49" s="46"/>
+      <c r="J49" s="46"/>
+      <c r="K49" s="46"/>
+      <c r="L49" s="47"/>
+      <c r="M49" s="45"/>
+      <c r="N49" s="46"/>
+      <c r="O49" s="46"/>
+      <c r="P49" s="47"/>
+      <c r="Q49" s="45"/>
+      <c r="R49" s="46"/>
+      <c r="S49" s="46"/>
+      <c r="T49" s="46"/>
+      <c r="U49" s="47"/>
+      <c r="V49" s="45"/>
+      <c r="W49" s="46"/>
+      <c r="X49" s="46"/>
+      <c r="Y49" s="46"/>
+      <c r="Z49" s="47"/>
+      <c r="AA49" s="45"/>
+      <c r="AB49" s="46"/>
+      <c r="AC49" s="46"/>
+      <c r="AD49" s="46"/>
+      <c r="AE49" s="48"/>
       <c r="AF49" s="16"/>
     </row>
     <row r="50" spans="1:32" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="18"/>
-      <c r="B50" s="50"/>
-      <c r="C50" s="51"/>
-      <c r="D50" s="51"/>
-      <c r="E50" s="51"/>
-      <c r="F50" s="51"/>
-      <c r="G50" s="51"/>
-      <c r="H50" s="51"/>
-      <c r="I50" s="51"/>
-      <c r="J50" s="51"/>
-      <c r="K50" s="51"/>
-      <c r="L50" s="51"/>
-      <c r="M50" s="51"/>
-      <c r="N50" s="51"/>
-      <c r="O50" s="51"/>
-      <c r="P50" s="51"/>
-      <c r="Q50" s="51"/>
-      <c r="R50" s="51"/>
-      <c r="S50" s="51"/>
-      <c r="T50" s="51"/>
-      <c r="U50" s="51"/>
-      <c r="V50" s="51"/>
-      <c r="W50" s="51"/>
-      <c r="X50" s="51"/>
-      <c r="Y50" s="51"/>
-      <c r="Z50" s="51"/>
-      <c r="AA50" s="51"/>
-      <c r="AB50" s="51"/>
-      <c r="AC50" s="51"/>
-      <c r="AD50" s="51"/>
-      <c r="AE50" s="52"/>
+      <c r="B50" s="49"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
+      <c r="E50" s="50"/>
+      <c r="F50" s="50"/>
+      <c r="G50" s="50"/>
+      <c r="H50" s="50"/>
+      <c r="I50" s="50"/>
+      <c r="J50" s="50"/>
+      <c r="K50" s="50"/>
+      <c r="L50" s="50"/>
+      <c r="M50" s="50"/>
+      <c r="N50" s="50"/>
+      <c r="O50" s="50"/>
+      <c r="P50" s="50"/>
+      <c r="Q50" s="50"/>
+      <c r="R50" s="50"/>
+      <c r="S50" s="50"/>
+      <c r="T50" s="50"/>
+      <c r="U50" s="50"/>
+      <c r="V50" s="50"/>
+      <c r="W50" s="50"/>
+      <c r="X50" s="50"/>
+      <c r="Y50" s="50"/>
+      <c r="Z50" s="50"/>
+      <c r="AA50" s="50"/>
+      <c r="AB50" s="50"/>
+      <c r="AC50" s="50"/>
+      <c r="AD50" s="50"/>
+      <c r="AE50" s="51"/>
       <c r="AF50" s="16"/>
     </row>
     <row r="51" spans="1:32" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="50"/>
-      <c r="B51" s="51"/>
-      <c r="C51" s="51"/>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51"/>
-      <c r="F51" s="51"/>
-      <c r="G51" s="51"/>
-      <c r="H51" s="51"/>
-      <c r="I51" s="51"/>
-      <c r="J51" s="51"/>
-      <c r="K51" s="51"/>
-      <c r="L51" s="51"/>
-      <c r="M51" s="51"/>
-      <c r="N51" s="51"/>
-      <c r="O51" s="51"/>
-      <c r="P51" s="51"/>
-      <c r="Q51" s="51"/>
-      <c r="R51" s="51"/>
-      <c r="S51" s="51"/>
-      <c r="T51" s="51"/>
-      <c r="U51" s="51"/>
-      <c r="V51" s="51"/>
-      <c r="W51" s="51"/>
-      <c r="X51" s="51"/>
-      <c r="Y51" s="51"/>
-      <c r="Z51" s="51"/>
-      <c r="AA51" s="51"/>
-      <c r="AB51" s="51"/>
-      <c r="AC51" s="51"/>
-      <c r="AD51" s="51"/>
-      <c r="AE51" s="51"/>
-      <c r="AF51" s="52"/>
+      <c r="A51" s="49"/>
+      <c r="B51" s="50"/>
+      <c r="C51" s="50"/>
+      <c r="D51" s="50"/>
+      <c r="E51" s="50"/>
+      <c r="F51" s="50"/>
+      <c r="G51" s="50"/>
+      <c r="H51" s="50"/>
+      <c r="I51" s="50"/>
+      <c r="J51" s="50"/>
+      <c r="K51" s="50"/>
+      <c r="L51" s="50"/>
+      <c r="M51" s="50"/>
+      <c r="N51" s="50"/>
+      <c r="O51" s="50"/>
+      <c r="P51" s="50"/>
+      <c r="Q51" s="50"/>
+      <c r="R51" s="50"/>
+      <c r="S51" s="50"/>
+      <c r="T51" s="50"/>
+      <c r="U51" s="50"/>
+      <c r="V51" s="50"/>
+      <c r="W51" s="50"/>
+      <c r="X51" s="50"/>
+      <c r="Y51" s="50"/>
+      <c r="Z51" s="50"/>
+      <c r="AA51" s="50"/>
+      <c r="AB51" s="50"/>
+      <c r="AC51" s="50"/>
+      <c r="AD51" s="50"/>
+      <c r="AE51" s="50"/>
+      <c r="AF51" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="59">
@@ -2866,7 +2853,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="61" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="63" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;L&amp;1#&amp;"Calibri"&amp;8&amp;K000000Sensitivity: LNT Construction Internal Use</oddFooter>
   </headerFooter>
@@ -2905,164 +2892,164 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="70.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="98" t="e" vm="1">
+      <c r="A1" s="99" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="95" t="s">
+      <c r="B1" s="99"/>
+      <c r="C1" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95" t="str">
+      <c r="D1" s="96"/>
+      <c r="E1" s="96" t="str">
         <f>"PROJECT : "&amp;Cover!F36</f>
-        <v>PROJECT : 0</v>
-      </c>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="95" t="s">
+        <v xml:space="preserve">PROJECT : </v>
+      </c>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="95"/>
-      <c r="S1" s="95"/>
-      <c r="T1" s="95"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
     </row>
     <row r="2" spans="1:20" ht="70.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="95">
+      <c r="B2" s="100"/>
+      <c r="C2" s="96" t="str">
         <f>_xlfn.SINGLE(Cover!F34)</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96" t="str">
         <f>"DOCUMENT NAME: "&amp;Cover!J39</f>
         <v xml:space="preserve">DOCUMENT NAME: INSTRUMENT LIST FOR </v>
       </c>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95" t="str">
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="96"/>
+      <c r="J2" s="96"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="96"/>
+      <c r="M2" s="96"/>
+      <c r="N2" s="96"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="96" t="str">
         <f>"DATE : "&amp;Cover!H40</f>
         <v>DATE : 00-01-00</v>
       </c>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="R2" s="96"/>
+      <c r="S2" s="96"/>
+      <c r="T2" s="96"/>
     </row>
     <row r="3" spans="1:20" ht="70.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="99" t="s">
+      <c r="A3" s="100" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="95">
+      <c r="B3" s="100"/>
+      <c r="C3" s="96" t="str">
         <f>_xlfn.SINGLE(Cover!F35)</f>
-        <v>0</v>
-      </c>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96" t="str">
         <f>"DOCUMENT NO:  "&amp;_xlfn.CONCAT(Cover!D44:AA44)&amp;"_ Rev. "&amp;Cover!AE44</f>
         <v>DOCUMENT NO:  _ Rev. 0</v>
       </c>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="95"/>
-      <c r="L3" s="95"/>
-      <c r="M3" s="95"/>
-      <c r="N3" s="95"/>
-      <c r="O3" s="95"/>
-      <c r="P3" s="95"/>
-      <c r="Q3" s="95" t="s">
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="96"/>
+      <c r="L3" s="96"/>
+      <c r="M3" s="96"/>
+      <c r="N3" s="96"/>
+      <c r="O3" s="96"/>
+      <c r="P3" s="96"/>
+      <c r="Q3" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="95"/>
-      <c r="S3" s="95"/>
-      <c r="T3" s="95"/>
+      <c r="R3" s="96"/>
+      <c r="S3" s="96"/>
+      <c r="T3" s="96"/>
     </row>
     <row r="4" spans="1:20" ht="46.8" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="96" t="s">
+      <c r="A4" s="97" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="96" t="s">
+      <c r="B4" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="96" t="s">
+      <c r="C4" s="97" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="96" t="s">
+      <c r="D4" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="96" t="s">
+      <c r="E4" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="96" t="s">
+      <c r="F4" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="96" t="s">
+      <c r="G4" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="96" t="s">
+      <c r="H4" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="96"/>
-      <c r="J4" s="96" t="s">
+      <c r="I4" s="97"/>
+      <c r="J4" s="97" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="96" t="s">
+      <c r="K4" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="96"/>
-      <c r="M4" s="96"/>
-      <c r="N4" s="96" t="s">
+      <c r="L4" s="97"/>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="96"/>
-      <c r="P4" s="96"/>
-      <c r="Q4" s="96" t="s">
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="R4" s="96" t="s">
+      <c r="R4" s="97" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="96" t="s">
+      <c r="S4" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="T4" s="96" t="s">
+      <c r="T4" s="97" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="46.8" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="96"/>
-      <c r="B5" s="96"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="96"/>
-      <c r="E5" s="96"/>
-      <c r="F5" s="96"/>
-      <c r="G5" s="96"/>
-      <c r="H5" s="96"/>
-      <c r="I5" s="96"/>
-      <c r="J5" s="96"/>
+      <c r="A5" s="97"/>
+      <c r="B5" s="97"/>
+      <c r="C5" s="97"/>
+      <c r="D5" s="97"/>
+      <c r="E5" s="97"/>
+      <c r="F5" s="97"/>
+      <c r="G5" s="97"/>
+      <c r="H5" s="97"/>
+      <c r="I5" s="97"/>
+      <c r="J5" s="97"/>
       <c r="K5" s="11" t="s">
         <v>18</v>
       </c>
@@ -3081,10 +3068,10 @@
       <c r="P5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="Q5" s="96"/>
-      <c r="R5" s="96"/>
-      <c r="S5" s="96"/>
-      <c r="T5" s="96"/>
+      <c r="Q5" s="97"/>
+      <c r="R5" s="97"/>
+      <c r="S5" s="97"/>
+      <c r="T5" s="97"/>
     </row>
     <row r="6" spans="1:20" ht="46.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
@@ -3094,8 +3081,8 @@
       <c r="E6" s="4"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="97"/>
-      <c r="I6" s="97"/>
+      <c r="H6" s="98"/>
+      <c r="I6" s="98"/>
       <c r="J6" s="3"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -3116,8 +3103,8 @@
       <c r="E7" s="4"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="94"/>
-      <c r="I7" s="94"/>
+      <c r="H7" s="95"/>
+      <c r="I7" s="95"/>
       <c r="J7" s="3"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
@@ -3138,8 +3125,8 @@
       <c r="E8" s="4"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="94"/>
-      <c r="I8" s="94"/>
+      <c r="H8" s="95"/>
+      <c r="I8" s="95"/>
       <c r="J8" s="3"/>
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
@@ -3160,8 +3147,8 @@
       <c r="E9" s="4"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="94"/>
-      <c r="I9" s="94"/>
+      <c r="H9" s="95"/>
+      <c r="I9" s="95"/>
       <c r="J9" s="3"/>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
@@ -3182,8 +3169,8 @@
       <c r="E10" s="4"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="94"/>
-      <c r="I10" s="94"/>
+      <c r="H10" s="95"/>
+      <c r="I10" s="95"/>
       <c r="J10" s="3"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
@@ -3204,8 +3191,8 @@
       <c r="E11" s="4"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="94"/>
-      <c r="I11" s="94"/>
+      <c r="H11" s="95"/>
+      <c r="I11" s="95"/>
       <c r="J11" s="3"/>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
@@ -3226,8 +3213,8 @@
       <c r="E12" s="4"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="94"/>
-      <c r="I12" s="94"/>
+      <c r="H12" s="95"/>
+      <c r="I12" s="95"/>
       <c r="J12" s="3"/>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
@@ -3248,8 +3235,8 @@
       <c r="E13" s="4"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="94"/>
-      <c r="I13" s="94"/>
+      <c r="H13" s="95"/>
+      <c r="I13" s="95"/>
       <c r="J13" s="3"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
@@ -3270,8 +3257,8 @@
       <c r="E14" s="4"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="94"/>
-      <c r="I14" s="94"/>
+      <c r="H14" s="95"/>
+      <c r="I14" s="95"/>
       <c r="J14" s="3"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>

</xml_diff>